<commit_message>
Fix YouTube autoplay: default to muted to comply with browser policies
</commit_message>
<xml_diff>
--- a/DANH SÁCH THÍ SINH.xlsx
+++ b/DANH SÁCH THÍ SINH.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="E:\TAO UNG DUNG\GAME RUNG CHUONG VANG\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{2BA9C308-7C97-4F7A-9E27-1686078AE4A3}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{62F305C8-A646-48B2-B80F-010DA8B15A48}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-98" yWindow="-98" windowWidth="20715" windowHeight="13155" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -28,7 +28,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="132" uniqueCount="131">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="196" uniqueCount="195">
   <si>
     <t>SBD</t>
   </si>
@@ -421,6 +421,198 @@
   </si>
   <si>
     <t>NGUYỄN VĂN NHÀN</t>
+  </si>
+  <si>
+    <t>01</t>
+  </si>
+  <si>
+    <t>02</t>
+  </si>
+  <si>
+    <t>03</t>
+  </si>
+  <si>
+    <t>04</t>
+  </si>
+  <si>
+    <t>05</t>
+  </si>
+  <si>
+    <t>06</t>
+  </si>
+  <si>
+    <t>07</t>
+  </si>
+  <si>
+    <t>08</t>
+  </si>
+  <si>
+    <t>09</t>
+  </si>
+  <si>
+    <t>10</t>
+  </si>
+  <si>
+    <t>11</t>
+  </si>
+  <si>
+    <t>12</t>
+  </si>
+  <si>
+    <t>13</t>
+  </si>
+  <si>
+    <t>14</t>
+  </si>
+  <si>
+    <t>15</t>
+  </si>
+  <si>
+    <t>16</t>
+  </si>
+  <si>
+    <t>17</t>
+  </si>
+  <si>
+    <t>18</t>
+  </si>
+  <si>
+    <t>19</t>
+  </si>
+  <si>
+    <t>20</t>
+  </si>
+  <si>
+    <t>21</t>
+  </si>
+  <si>
+    <t>22</t>
+  </si>
+  <si>
+    <t>23</t>
+  </si>
+  <si>
+    <t>24</t>
+  </si>
+  <si>
+    <t>25</t>
+  </si>
+  <si>
+    <t>26</t>
+  </si>
+  <si>
+    <t>27</t>
+  </si>
+  <si>
+    <t>28</t>
+  </si>
+  <si>
+    <t>29</t>
+  </si>
+  <si>
+    <t>30</t>
+  </si>
+  <si>
+    <t>31</t>
+  </si>
+  <si>
+    <t>32</t>
+  </si>
+  <si>
+    <t>33</t>
+  </si>
+  <si>
+    <t>34</t>
+  </si>
+  <si>
+    <t>35</t>
+  </si>
+  <si>
+    <t>36</t>
+  </si>
+  <si>
+    <t>37</t>
+  </si>
+  <si>
+    <t>38</t>
+  </si>
+  <si>
+    <t>39</t>
+  </si>
+  <si>
+    <t>40</t>
+  </si>
+  <si>
+    <t>41</t>
+  </si>
+  <si>
+    <t>42</t>
+  </si>
+  <si>
+    <t>43</t>
+  </si>
+  <si>
+    <t>44</t>
+  </si>
+  <si>
+    <t>45</t>
+  </si>
+  <si>
+    <t>46</t>
+  </si>
+  <si>
+    <t>47</t>
+  </si>
+  <si>
+    <t>48</t>
+  </si>
+  <si>
+    <t>49</t>
+  </si>
+  <si>
+    <t>50</t>
+  </si>
+  <si>
+    <t>51</t>
+  </si>
+  <si>
+    <t>52</t>
+  </si>
+  <si>
+    <t>53</t>
+  </si>
+  <si>
+    <t>54</t>
+  </si>
+  <si>
+    <t>55</t>
+  </si>
+  <si>
+    <t>56</t>
+  </si>
+  <si>
+    <t>57</t>
+  </si>
+  <si>
+    <t>58</t>
+  </si>
+  <si>
+    <t>59</t>
+  </si>
+  <si>
+    <t>60</t>
+  </si>
+  <si>
+    <t>61</t>
+  </si>
+  <si>
+    <t>62</t>
+  </si>
+  <si>
+    <t>63</t>
+  </si>
+  <si>
+    <t>64</t>
   </si>
 </sst>
 </file>
@@ -462,8 +654,9 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="1">
+  <cellXfs count="2">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
+    <xf numFmtId="49" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -747,11 +940,12 @@
   <dimension ref="A1:D65"/>
   <sheetFormatPr defaultRowHeight="14.25" x14ac:dyDescent="0.45"/>
   <cols>
+    <col min="1" max="1" width="9.06640625" style="1"/>
     <col min="2" max="2" width="18.46484375" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:4" x14ac:dyDescent="0.45">
-      <c r="A1" t="s">
+      <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
       <c r="B1" t="s">
@@ -765,8 +959,8 @@
       </c>
     </row>
     <row r="2" spans="1:4" x14ac:dyDescent="0.45">
-      <c r="A2">
-        <v>1</v>
+      <c r="A2" s="1" t="s">
+        <v>131</v>
       </c>
       <c r="B2" t="s">
         <v>127</v>
@@ -779,8 +973,8 @@
       </c>
     </row>
     <row r="3" spans="1:4" x14ac:dyDescent="0.45">
-      <c r="A3">
-        <v>2</v>
+      <c r="A3" s="1" t="s">
+        <v>132</v>
       </c>
       <c r="B3" t="s">
         <v>128</v>
@@ -793,8 +987,8 @@
       </c>
     </row>
     <row r="4" spans="1:4" x14ac:dyDescent="0.45">
-      <c r="A4">
-        <v>3</v>
+      <c r="A4" s="1" t="s">
+        <v>133</v>
       </c>
       <c r="B4" t="s">
         <v>129</v>
@@ -807,8 +1001,8 @@
       </c>
     </row>
     <row r="5" spans="1:4" x14ac:dyDescent="0.45">
-      <c r="A5">
-        <v>4</v>
+      <c r="A5" s="1" t="s">
+        <v>134</v>
       </c>
       <c r="B5" t="s">
         <v>21</v>
@@ -821,8 +1015,8 @@
       </c>
     </row>
     <row r="6" spans="1:4" x14ac:dyDescent="0.45">
-      <c r="A6">
-        <v>5</v>
+      <c r="A6" s="1" t="s">
+        <v>135</v>
       </c>
       <c r="B6" t="s">
         <v>22</v>
@@ -835,8 +1029,8 @@
       </c>
     </row>
     <row r="7" spans="1:4" x14ac:dyDescent="0.45">
-      <c r="A7">
-        <v>6</v>
+      <c r="A7" s="1" t="s">
+        <v>136</v>
       </c>
       <c r="B7" t="s">
         <v>23</v>
@@ -849,8 +1043,8 @@
       </c>
     </row>
     <row r="8" spans="1:4" x14ac:dyDescent="0.45">
-      <c r="A8">
-        <v>7</v>
+      <c r="A8" s="1" t="s">
+        <v>137</v>
       </c>
       <c r="B8" t="s">
         <v>24</v>
@@ -863,8 +1057,8 @@
       </c>
     </row>
     <row r="9" spans="1:4" x14ac:dyDescent="0.45">
-      <c r="A9">
-        <v>8</v>
+      <c r="A9" s="1" t="s">
+        <v>138</v>
       </c>
       <c r="B9" t="s">
         <v>25</v>
@@ -877,8 +1071,8 @@
       </c>
     </row>
     <row r="10" spans="1:4" x14ac:dyDescent="0.45">
-      <c r="A10">
-        <v>9</v>
+      <c r="A10" s="1" t="s">
+        <v>139</v>
       </c>
       <c r="B10" t="s">
         <v>26</v>
@@ -891,8 +1085,8 @@
       </c>
     </row>
     <row r="11" spans="1:4" x14ac:dyDescent="0.45">
-      <c r="A11">
-        <v>10</v>
+      <c r="A11" s="1" t="s">
+        <v>140</v>
       </c>
       <c r="B11" t="s">
         <v>129</v>
@@ -905,8 +1099,8 @@
       </c>
     </row>
     <row r="12" spans="1:4" x14ac:dyDescent="0.45">
-      <c r="A12">
-        <v>11</v>
+      <c r="A12" s="1" t="s">
+        <v>141</v>
       </c>
       <c r="B12" t="s">
         <v>130</v>
@@ -919,8 +1113,8 @@
       </c>
     </row>
     <row r="13" spans="1:4" x14ac:dyDescent="0.45">
-      <c r="A13">
-        <v>12</v>
+      <c r="A13" s="1" t="s">
+        <v>142</v>
       </c>
       <c r="B13" t="s">
         <v>27</v>
@@ -933,8 +1127,8 @@
       </c>
     </row>
     <row r="14" spans="1:4" x14ac:dyDescent="0.45">
-      <c r="A14">
-        <v>13</v>
+      <c r="A14" s="1" t="s">
+        <v>143</v>
       </c>
       <c r="B14" t="s">
         <v>28</v>
@@ -947,8 +1141,8 @@
       </c>
     </row>
     <row r="15" spans="1:4" x14ac:dyDescent="0.45">
-      <c r="A15">
-        <v>14</v>
+      <c r="A15" s="1" t="s">
+        <v>144</v>
       </c>
       <c r="B15" t="s">
         <v>29</v>
@@ -961,8 +1155,8 @@
       </c>
     </row>
     <row r="16" spans="1:4" x14ac:dyDescent="0.45">
-      <c r="A16">
-        <v>15</v>
+      <c r="A16" s="1" t="s">
+        <v>145</v>
       </c>
       <c r="B16" t="s">
         <v>30</v>
@@ -975,8 +1169,8 @@
       </c>
     </row>
     <row r="17" spans="1:4" x14ac:dyDescent="0.45">
-      <c r="A17">
-        <v>16</v>
+      <c r="A17" s="1" t="s">
+        <v>146</v>
       </c>
       <c r="B17" t="s">
         <v>5</v>
@@ -989,8 +1183,8 @@
       </c>
     </row>
     <row r="18" spans="1:4" x14ac:dyDescent="0.45">
-      <c r="A18">
-        <v>17</v>
+      <c r="A18" s="1" t="s">
+        <v>147</v>
       </c>
       <c r="B18" t="s">
         <v>6</v>
@@ -1003,8 +1197,8 @@
       </c>
     </row>
     <row r="19" spans="1:4" x14ac:dyDescent="0.45">
-      <c r="A19">
-        <v>18</v>
+      <c r="A19" s="1" t="s">
+        <v>148</v>
       </c>
       <c r="B19" t="s">
         <v>7</v>
@@ -1017,8 +1211,8 @@
       </c>
     </row>
     <row r="20" spans="1:4" x14ac:dyDescent="0.45">
-      <c r="A20">
-        <v>19</v>
+      <c r="A20" s="1" t="s">
+        <v>149</v>
       </c>
       <c r="B20" t="s">
         <v>8</v>
@@ -1031,8 +1225,8 @@
       </c>
     </row>
     <row r="21" spans="1:4" x14ac:dyDescent="0.45">
-      <c r="A21">
-        <v>20</v>
+      <c r="A21" s="1" t="s">
+        <v>150</v>
       </c>
       <c r="B21" t="s">
         <v>9</v>
@@ -1045,8 +1239,8 @@
       </c>
     </row>
     <row r="22" spans="1:4" x14ac:dyDescent="0.45">
-      <c r="A22">
-        <v>21</v>
+      <c r="A22" s="1" t="s">
+        <v>151</v>
       </c>
       <c r="B22" t="s">
         <v>10</v>
@@ -1059,8 +1253,8 @@
       </c>
     </row>
     <row r="23" spans="1:4" x14ac:dyDescent="0.45">
-      <c r="A23">
-        <v>22</v>
+      <c r="A23" s="1" t="s">
+        <v>152</v>
       </c>
       <c r="B23" t="s">
         <v>11</v>
@@ -1073,8 +1267,8 @@
       </c>
     </row>
     <row r="24" spans="1:4" x14ac:dyDescent="0.45">
-      <c r="A24">
-        <v>23</v>
+      <c r="A24" s="1" t="s">
+        <v>153</v>
       </c>
       <c r="B24" t="s">
         <v>12</v>
@@ -1087,8 +1281,8 @@
       </c>
     </row>
     <row r="25" spans="1:4" x14ac:dyDescent="0.45">
-      <c r="A25">
-        <v>24</v>
+      <c r="A25" s="1" t="s">
+        <v>154</v>
       </c>
       <c r="B25" t="s">
         <v>13</v>
@@ -1101,8 +1295,8 @@
       </c>
     </row>
     <row r="26" spans="1:4" x14ac:dyDescent="0.45">
-      <c r="A26">
-        <v>25</v>
+      <c r="A26" s="1" t="s">
+        <v>155</v>
       </c>
       <c r="B26" t="s">
         <v>14</v>
@@ -1115,8 +1309,8 @@
       </c>
     </row>
     <row r="27" spans="1:4" x14ac:dyDescent="0.45">
-      <c r="A27">
-        <v>26</v>
+      <c r="A27" s="1" t="s">
+        <v>156</v>
       </c>
       <c r="B27" t="s">
         <v>15</v>
@@ -1129,8 +1323,8 @@
       </c>
     </row>
     <row r="28" spans="1:4" x14ac:dyDescent="0.45">
-      <c r="A28">
-        <v>27</v>
+      <c r="A28" s="1" t="s">
+        <v>157</v>
       </c>
       <c r="B28" t="s">
         <v>16</v>
@@ -1143,8 +1337,8 @@
       </c>
     </row>
     <row r="29" spans="1:4" x14ac:dyDescent="0.45">
-      <c r="A29">
-        <v>28</v>
+      <c r="A29" s="1" t="s">
+        <v>158</v>
       </c>
       <c r="B29" t="s">
         <v>17</v>
@@ -1157,8 +1351,8 @@
       </c>
     </row>
     <row r="30" spans="1:4" x14ac:dyDescent="0.45">
-      <c r="A30">
-        <v>29</v>
+      <c r="A30" s="1" t="s">
+        <v>159</v>
       </c>
       <c r="B30" t="s">
         <v>18</v>
@@ -1171,8 +1365,8 @@
       </c>
     </row>
     <row r="31" spans="1:4" x14ac:dyDescent="0.45">
-      <c r="A31">
-        <v>30</v>
+      <c r="A31" s="1" t="s">
+        <v>160</v>
       </c>
       <c r="B31" t="s">
         <v>19</v>
@@ -1185,8 +1379,8 @@
       </c>
     </row>
     <row r="32" spans="1:4" x14ac:dyDescent="0.45">
-      <c r="A32">
-        <v>31</v>
+      <c r="A32" s="1" t="s">
+        <v>161</v>
       </c>
       <c r="B32" t="s">
         <v>20</v>
@@ -1199,8 +1393,8 @@
       </c>
     </row>
     <row r="33" spans="1:4" x14ac:dyDescent="0.45">
-      <c r="A33">
-        <v>32</v>
+      <c r="A33" s="1" t="s">
+        <v>162</v>
       </c>
       <c r="B33" t="s">
         <v>31</v>
@@ -1213,8 +1407,8 @@
       </c>
     </row>
     <row r="34" spans="1:4" x14ac:dyDescent="0.45">
-      <c r="A34">
-        <v>33</v>
+      <c r="A34" s="1" t="s">
+        <v>163</v>
       </c>
       <c r="B34" t="s">
         <v>32</v>
@@ -1227,8 +1421,8 @@
       </c>
     </row>
     <row r="35" spans="1:4" x14ac:dyDescent="0.45">
-      <c r="A35">
-        <v>34</v>
+      <c r="A35" s="1" t="s">
+        <v>164</v>
       </c>
       <c r="B35" t="s">
         <v>33</v>
@@ -1241,8 +1435,8 @@
       </c>
     </row>
     <row r="36" spans="1:4" x14ac:dyDescent="0.45">
-      <c r="A36">
-        <v>35</v>
+      <c r="A36" s="1" t="s">
+        <v>165</v>
       </c>
       <c r="B36" t="s">
         <v>34</v>
@@ -1255,8 +1449,8 @@
       </c>
     </row>
     <row r="37" spans="1:4" x14ac:dyDescent="0.45">
-      <c r="A37">
-        <v>36</v>
+      <c r="A37" s="1" t="s">
+        <v>166</v>
       </c>
       <c r="B37" t="s">
         <v>35</v>
@@ -1269,8 +1463,8 @@
       </c>
     </row>
     <row r="38" spans="1:4" x14ac:dyDescent="0.45">
-      <c r="A38">
-        <v>37</v>
+      <c r="A38" s="1" t="s">
+        <v>167</v>
       </c>
       <c r="B38" t="s">
         <v>36</v>
@@ -1283,8 +1477,8 @@
       </c>
     </row>
     <row r="39" spans="1:4" x14ac:dyDescent="0.45">
-      <c r="A39">
-        <v>38</v>
+      <c r="A39" s="1" t="s">
+        <v>168</v>
       </c>
       <c r="B39" t="s">
         <v>37</v>
@@ -1297,8 +1491,8 @@
       </c>
     </row>
     <row r="40" spans="1:4" x14ac:dyDescent="0.45">
-      <c r="A40">
-        <v>39</v>
+      <c r="A40" s="1" t="s">
+        <v>169</v>
       </c>
       <c r="B40" t="s">
         <v>38</v>
@@ -1311,8 +1505,8 @@
       </c>
     </row>
     <row r="41" spans="1:4" x14ac:dyDescent="0.45">
-      <c r="A41">
-        <v>40</v>
+      <c r="A41" s="1" t="s">
+        <v>170</v>
       </c>
       <c r="B41" t="s">
         <v>39</v>
@@ -1325,8 +1519,8 @@
       </c>
     </row>
     <row r="42" spans="1:4" x14ac:dyDescent="0.45">
-      <c r="A42">
-        <v>41</v>
+      <c r="A42" s="1" t="s">
+        <v>171</v>
       </c>
       <c r="B42" t="s">
         <v>40</v>
@@ -1339,8 +1533,8 @@
       </c>
     </row>
     <row r="43" spans="1:4" x14ac:dyDescent="0.45">
-      <c r="A43">
-        <v>42</v>
+      <c r="A43" s="1" t="s">
+        <v>172</v>
       </c>
       <c r="B43" t="s">
         <v>41</v>
@@ -1353,8 +1547,8 @@
       </c>
     </row>
     <row r="44" spans="1:4" x14ac:dyDescent="0.45">
-      <c r="A44">
-        <v>43</v>
+      <c r="A44" s="1" t="s">
+        <v>173</v>
       </c>
       <c r="B44" t="s">
         <v>42</v>
@@ -1367,8 +1561,8 @@
       </c>
     </row>
     <row r="45" spans="1:4" x14ac:dyDescent="0.45">
-      <c r="A45">
-        <v>44</v>
+      <c r="A45" s="1" t="s">
+        <v>174</v>
       </c>
       <c r="B45" t="s">
         <v>43</v>
@@ -1381,8 +1575,8 @@
       </c>
     </row>
     <row r="46" spans="1:4" x14ac:dyDescent="0.45">
-      <c r="A46">
-        <v>45</v>
+      <c r="A46" s="1" t="s">
+        <v>175</v>
       </c>
       <c r="B46" t="s">
         <v>44</v>
@@ -1395,8 +1589,8 @@
       </c>
     </row>
     <row r="47" spans="1:4" x14ac:dyDescent="0.45">
-      <c r="A47">
-        <v>46</v>
+      <c r="A47" s="1" t="s">
+        <v>176</v>
       </c>
       <c r="B47" t="s">
         <v>45</v>
@@ -1409,8 +1603,8 @@
       </c>
     </row>
     <row r="48" spans="1:4" x14ac:dyDescent="0.45">
-      <c r="A48">
-        <v>47</v>
+      <c r="A48" s="1" t="s">
+        <v>177</v>
       </c>
       <c r="B48" t="s">
         <v>46</v>
@@ -1423,8 +1617,8 @@
       </c>
     </row>
     <row r="49" spans="1:4" x14ac:dyDescent="0.45">
-      <c r="A49">
-        <v>48</v>
+      <c r="A49" s="1" t="s">
+        <v>178</v>
       </c>
       <c r="B49" t="s">
         <v>47</v>
@@ -1437,8 +1631,8 @@
       </c>
     </row>
     <row r="50" spans="1:4" x14ac:dyDescent="0.45">
-      <c r="A50">
-        <v>49</v>
+      <c r="A50" s="1" t="s">
+        <v>179</v>
       </c>
       <c r="B50" t="s">
         <v>48</v>
@@ -1451,8 +1645,8 @@
       </c>
     </row>
     <row r="51" spans="1:4" x14ac:dyDescent="0.45">
-      <c r="A51">
-        <v>50</v>
+      <c r="A51" s="1" t="s">
+        <v>180</v>
       </c>
       <c r="B51" t="s">
         <v>49</v>
@@ -1465,8 +1659,8 @@
       </c>
     </row>
     <row r="52" spans="1:4" x14ac:dyDescent="0.45">
-      <c r="A52">
-        <v>51</v>
+      <c r="A52" s="1" t="s">
+        <v>181</v>
       </c>
       <c r="B52" t="s">
         <v>50</v>
@@ -1479,8 +1673,8 @@
       </c>
     </row>
     <row r="53" spans="1:4" x14ac:dyDescent="0.45">
-      <c r="A53">
-        <v>52</v>
+      <c r="A53" s="1" t="s">
+        <v>182</v>
       </c>
       <c r="B53" t="s">
         <v>51</v>
@@ -1493,8 +1687,8 @@
       </c>
     </row>
     <row r="54" spans="1:4" x14ac:dyDescent="0.45">
-      <c r="A54">
-        <v>53</v>
+      <c r="A54" s="1" t="s">
+        <v>183</v>
       </c>
       <c r="B54" t="s">
         <v>52</v>
@@ -1507,8 +1701,8 @@
       </c>
     </row>
     <row r="55" spans="1:4" x14ac:dyDescent="0.45">
-      <c r="A55">
-        <v>54</v>
+      <c r="A55" s="1" t="s">
+        <v>184</v>
       </c>
       <c r="B55" t="s">
         <v>53</v>
@@ -1521,8 +1715,8 @@
       </c>
     </row>
     <row r="56" spans="1:4" x14ac:dyDescent="0.45">
-      <c r="A56">
-        <v>55</v>
+      <c r="A56" s="1" t="s">
+        <v>185</v>
       </c>
       <c r="B56" t="s">
         <v>54</v>
@@ -1535,8 +1729,8 @@
       </c>
     </row>
     <row r="57" spans="1:4" x14ac:dyDescent="0.45">
-      <c r="A57">
-        <v>56</v>
+      <c r="A57" s="1" t="s">
+        <v>186</v>
       </c>
       <c r="B57" t="s">
         <v>55</v>
@@ -1549,8 +1743,8 @@
       </c>
     </row>
     <row r="58" spans="1:4" x14ac:dyDescent="0.45">
-      <c r="A58">
-        <v>57</v>
+      <c r="A58" s="1" t="s">
+        <v>187</v>
       </c>
       <c r="B58" t="s">
         <v>56</v>
@@ -1563,8 +1757,8 @@
       </c>
     </row>
     <row r="59" spans="1:4" x14ac:dyDescent="0.45">
-      <c r="A59">
-        <v>58</v>
+      <c r="A59" s="1" t="s">
+        <v>188</v>
       </c>
       <c r="B59" t="s">
         <v>57</v>
@@ -1577,8 +1771,8 @@
       </c>
     </row>
     <row r="60" spans="1:4" x14ac:dyDescent="0.45">
-      <c r="A60">
-        <v>59</v>
+      <c r="A60" s="1" t="s">
+        <v>189</v>
       </c>
       <c r="B60" t="s">
         <v>58</v>
@@ -1591,8 +1785,8 @@
       </c>
     </row>
     <row r="61" spans="1:4" x14ac:dyDescent="0.45">
-      <c r="A61">
-        <v>60</v>
+      <c r="A61" s="1" t="s">
+        <v>190</v>
       </c>
       <c r="B61" t="s">
         <v>59</v>
@@ -1605,8 +1799,8 @@
       </c>
     </row>
     <row r="62" spans="1:4" x14ac:dyDescent="0.45">
-      <c r="A62">
-        <v>61</v>
+      <c r="A62" s="1" t="s">
+        <v>191</v>
       </c>
       <c r="B62" t="s">
         <v>60</v>
@@ -1619,8 +1813,8 @@
       </c>
     </row>
     <row r="63" spans="1:4" x14ac:dyDescent="0.45">
-      <c r="A63">
-        <v>62</v>
+      <c r="A63" s="1" t="s">
+        <v>192</v>
       </c>
       <c r="B63" t="s">
         <v>61</v>
@@ -1633,8 +1827,8 @@
       </c>
     </row>
     <row r="64" spans="1:4" x14ac:dyDescent="0.45">
-      <c r="A64">
-        <v>63</v>
+      <c r="A64" s="1" t="s">
+        <v>193</v>
       </c>
       <c r="B64" t="s">
         <v>62</v>
@@ -1647,8 +1841,8 @@
       </c>
     </row>
     <row r="65" spans="1:4" x14ac:dyDescent="0.45">
-      <c r="A65">
-        <v>64</v>
+      <c r="A65" s="1" t="s">
+        <v>194</v>
       </c>
       <c r="B65" t="s">
         <v>63</v>
@@ -1663,5 +1857,6 @@
   </sheetData>
   <phoneticPr fontId="1" type="noConversion"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <pageSetup paperSize="9" orientation="portrait" horizontalDpi="0" verticalDpi="0" r:id="rId1"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Layout: Media between question and options. Parsers: Auto-detect YouTube links. Admin: Clean up UI.
</commit_message>
<xml_diff>
--- a/DANH SÁCH THÍ SINH.xlsx
+++ b/DANH SÁCH THÍ SINH.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="E:\TAO UNG DUNG\GAME RUNG CHUONG VANG\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{62F305C8-A646-48B2-B80F-010DA8B15A48}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{973387B7-B8AD-4AA1-8988-8B6C796DCF03}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-98" yWindow="-98" windowWidth="20715" windowHeight="13155" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -28,7 +28,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="196" uniqueCount="195">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="260" uniqueCount="195">
   <si>
     <t>SBD</t>
   </si>
@@ -423,196 +423,196 @@
     <t>NGUYỄN VĂN NHÀN</t>
   </si>
   <si>
-    <t>01</t>
-  </si>
-  <si>
-    <t>02</t>
-  </si>
-  <si>
-    <t>03</t>
-  </si>
-  <si>
-    <t>04</t>
-  </si>
-  <si>
-    <t>05</t>
-  </si>
-  <si>
-    <t>06</t>
-  </si>
-  <si>
-    <t>07</t>
-  </si>
-  <si>
-    <t>08</t>
-  </si>
-  <si>
-    <t>09</t>
-  </si>
-  <si>
-    <t>10</t>
-  </si>
-  <si>
-    <t>11</t>
-  </si>
-  <si>
-    <t>12</t>
-  </si>
-  <si>
-    <t>13</t>
-  </si>
-  <si>
-    <t>14</t>
-  </si>
-  <si>
-    <t>15</t>
-  </si>
-  <si>
-    <t>16</t>
-  </si>
-  <si>
-    <t>17</t>
-  </si>
-  <si>
-    <t>18</t>
-  </si>
-  <si>
-    <t>19</t>
-  </si>
-  <si>
-    <t>20</t>
-  </si>
-  <si>
-    <t>21</t>
-  </si>
-  <si>
-    <t>22</t>
-  </si>
-  <si>
-    <t>23</t>
-  </si>
-  <si>
-    <t>24</t>
-  </si>
-  <si>
-    <t>25</t>
-  </si>
-  <si>
-    <t>26</t>
-  </si>
-  <si>
-    <t>27</t>
-  </si>
-  <si>
-    <t>28</t>
-  </si>
-  <si>
-    <t>29</t>
-  </si>
-  <si>
-    <t>30</t>
-  </si>
-  <si>
-    <t>31</t>
-  </si>
-  <si>
-    <t>32</t>
-  </si>
-  <si>
-    <t>33</t>
-  </si>
-  <si>
-    <t>34</t>
-  </si>
-  <si>
-    <t>35</t>
-  </si>
-  <si>
-    <t>36</t>
-  </si>
-  <si>
-    <t>37</t>
-  </si>
-  <si>
-    <t>38</t>
-  </si>
-  <si>
-    <t>39</t>
-  </si>
-  <si>
-    <t>40</t>
-  </si>
-  <si>
-    <t>41</t>
-  </si>
-  <si>
-    <t>42</t>
-  </si>
-  <si>
-    <t>43</t>
-  </si>
-  <si>
-    <t>44</t>
-  </si>
-  <si>
-    <t>45</t>
-  </si>
-  <si>
-    <t>46</t>
-  </si>
-  <si>
-    <t>47</t>
-  </si>
-  <si>
-    <t>48</t>
-  </si>
-  <si>
-    <t>49</t>
-  </si>
-  <si>
-    <t>50</t>
-  </si>
-  <si>
-    <t>51</t>
-  </si>
-  <si>
-    <t>52</t>
-  </si>
-  <si>
-    <t>53</t>
-  </si>
-  <si>
-    <t>54</t>
-  </si>
-  <si>
-    <t>55</t>
-  </si>
-  <si>
-    <t>56</t>
-  </si>
-  <si>
-    <t>57</t>
-  </si>
-  <si>
-    <t>58</t>
-  </si>
-  <si>
-    <t>59</t>
-  </si>
-  <si>
-    <t>60</t>
-  </si>
-  <si>
-    <t>61</t>
-  </si>
-  <si>
-    <t>62</t>
-  </si>
-  <si>
-    <t>63</t>
-  </si>
-  <si>
-    <t>64</t>
+    <t>101</t>
+  </si>
+  <si>
+    <t>102</t>
+  </si>
+  <si>
+    <t>103</t>
+  </si>
+  <si>
+    <t>104</t>
+  </si>
+  <si>
+    <t>105</t>
+  </si>
+  <si>
+    <t>106</t>
+  </si>
+  <si>
+    <t>107</t>
+  </si>
+  <si>
+    <t>108</t>
+  </si>
+  <si>
+    <t>109</t>
+  </si>
+  <si>
+    <t>110</t>
+  </si>
+  <si>
+    <t>111</t>
+  </si>
+  <si>
+    <t>112</t>
+  </si>
+  <si>
+    <t>113</t>
+  </si>
+  <si>
+    <t>114</t>
+  </si>
+  <si>
+    <t>115</t>
+  </si>
+  <si>
+    <t>116</t>
+  </si>
+  <si>
+    <t>117</t>
+  </si>
+  <si>
+    <t>118</t>
+  </si>
+  <si>
+    <t>119</t>
+  </si>
+  <si>
+    <t>120</t>
+  </si>
+  <si>
+    <t>121</t>
+  </si>
+  <si>
+    <t>122</t>
+  </si>
+  <si>
+    <t>123</t>
+  </si>
+  <si>
+    <t>124</t>
+  </si>
+  <si>
+    <t>125</t>
+  </si>
+  <si>
+    <t>126</t>
+  </si>
+  <si>
+    <t>127</t>
+  </si>
+  <si>
+    <t>128</t>
+  </si>
+  <si>
+    <t>129</t>
+  </si>
+  <si>
+    <t>130</t>
+  </si>
+  <si>
+    <t>131</t>
+  </si>
+  <si>
+    <t>132</t>
+  </si>
+  <si>
+    <t>133</t>
+  </si>
+  <si>
+    <t>134</t>
+  </si>
+  <si>
+    <t>135</t>
+  </si>
+  <si>
+    <t>136</t>
+  </si>
+  <si>
+    <t>137</t>
+  </si>
+  <si>
+    <t>138</t>
+  </si>
+  <si>
+    <t>139</t>
+  </si>
+  <si>
+    <t>140</t>
+  </si>
+  <si>
+    <t>141</t>
+  </si>
+  <si>
+    <t>142</t>
+  </si>
+  <si>
+    <t>143</t>
+  </si>
+  <si>
+    <t>144</t>
+  </si>
+  <si>
+    <t>145</t>
+  </si>
+  <si>
+    <t>146</t>
+  </si>
+  <si>
+    <t>147</t>
+  </si>
+  <si>
+    <t>148</t>
+  </si>
+  <si>
+    <t>149</t>
+  </si>
+  <si>
+    <t>150</t>
+  </si>
+  <si>
+    <t>151</t>
+  </si>
+  <si>
+    <t>152</t>
+  </si>
+  <si>
+    <t>153</t>
+  </si>
+  <si>
+    <t>154</t>
+  </si>
+  <si>
+    <t>155</t>
+  </si>
+  <si>
+    <t>156</t>
+  </si>
+  <si>
+    <t>157</t>
+  </si>
+  <si>
+    <t>158</t>
+  </si>
+  <si>
+    <t>159</t>
+  </si>
+  <si>
+    <t>160</t>
+  </si>
+  <si>
+    <t>161</t>
+  </si>
+  <si>
+    <t>162</t>
+  </si>
+  <si>
+    <t>163</t>
+  </si>
+  <si>
+    <t>164</t>
   </si>
 </sst>
 </file>
@@ -942,6 +942,7 @@
   <cols>
     <col min="1" max="1" width="9.06640625" style="1"/>
     <col min="2" max="2" width="18.46484375" customWidth="1"/>
+    <col min="4" max="4" width="9.06640625" style="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:4" x14ac:dyDescent="0.45">
@@ -954,7 +955,7 @@
       <c r="C1" t="s">
         <v>2</v>
       </c>
-      <c r="D1" t="s">
+      <c r="D1" s="1" t="s">
         <v>3</v>
       </c>
     </row>
@@ -968,8 +969,8 @@
       <c r="C2" t="s">
         <v>4</v>
       </c>
-      <c r="D2">
-        <v>1</v>
+      <c r="D2" s="1" t="s">
+        <v>131</v>
       </c>
     </row>
     <row r="3" spans="1:4" x14ac:dyDescent="0.45">
@@ -982,8 +983,8 @@
       <c r="C3" t="s">
         <v>64</v>
       </c>
-      <c r="D3">
-        <v>2</v>
+      <c r="D3" s="1" t="s">
+        <v>132</v>
       </c>
     </row>
     <row r="4" spans="1:4" x14ac:dyDescent="0.45">
@@ -996,8 +997,8 @@
       <c r="C4" t="s">
         <v>65</v>
       </c>
-      <c r="D4">
-        <v>3</v>
+      <c r="D4" s="1" t="s">
+        <v>133</v>
       </c>
     </row>
     <row r="5" spans="1:4" x14ac:dyDescent="0.45">
@@ -1010,8 +1011,8 @@
       <c r="C5" t="s">
         <v>66</v>
       </c>
-      <c r="D5">
-        <v>4</v>
+      <c r="D5" s="1" t="s">
+        <v>134</v>
       </c>
     </row>
     <row r="6" spans="1:4" x14ac:dyDescent="0.45">
@@ -1024,8 +1025,8 @@
       <c r="C6" t="s">
         <v>67</v>
       </c>
-      <c r="D6">
-        <v>5</v>
+      <c r="D6" s="1" t="s">
+        <v>135</v>
       </c>
     </row>
     <row r="7" spans="1:4" x14ac:dyDescent="0.45">
@@ -1038,8 +1039,8 @@
       <c r="C7" t="s">
         <v>68</v>
       </c>
-      <c r="D7">
-        <v>6</v>
+      <c r="D7" s="1" t="s">
+        <v>136</v>
       </c>
     </row>
     <row r="8" spans="1:4" x14ac:dyDescent="0.45">
@@ -1052,8 +1053,8 @@
       <c r="C8" t="s">
         <v>69</v>
       </c>
-      <c r="D8">
-        <v>7</v>
+      <c r="D8" s="1" t="s">
+        <v>137</v>
       </c>
     </row>
     <row r="9" spans="1:4" x14ac:dyDescent="0.45">
@@ -1066,8 +1067,8 @@
       <c r="C9" t="s">
         <v>70</v>
       </c>
-      <c r="D9">
-        <v>8</v>
+      <c r="D9" s="1" t="s">
+        <v>138</v>
       </c>
     </row>
     <row r="10" spans="1:4" x14ac:dyDescent="0.45">
@@ -1080,8 +1081,8 @@
       <c r="C10" t="s">
         <v>71</v>
       </c>
-      <c r="D10">
-        <v>9</v>
+      <c r="D10" s="1" t="s">
+        <v>139</v>
       </c>
     </row>
     <row r="11" spans="1:4" x14ac:dyDescent="0.45">
@@ -1094,8 +1095,8 @@
       <c r="C11" t="s">
         <v>72</v>
       </c>
-      <c r="D11">
-        <v>10</v>
+      <c r="D11" s="1" t="s">
+        <v>140</v>
       </c>
     </row>
     <row r="12" spans="1:4" x14ac:dyDescent="0.45">
@@ -1108,8 +1109,8 @@
       <c r="C12" t="s">
         <v>73</v>
       </c>
-      <c r="D12">
-        <v>11</v>
+      <c r="D12" s="1" t="s">
+        <v>141</v>
       </c>
     </row>
     <row r="13" spans="1:4" x14ac:dyDescent="0.45">
@@ -1122,8 +1123,8 @@
       <c r="C13" t="s">
         <v>74</v>
       </c>
-      <c r="D13">
-        <v>12</v>
+      <c r="D13" s="1" t="s">
+        <v>142</v>
       </c>
     </row>
     <row r="14" spans="1:4" x14ac:dyDescent="0.45">
@@ -1136,8 +1137,8 @@
       <c r="C14" t="s">
         <v>75</v>
       </c>
-      <c r="D14">
-        <v>13</v>
+      <c r="D14" s="1" t="s">
+        <v>143</v>
       </c>
     </row>
     <row r="15" spans="1:4" x14ac:dyDescent="0.45">
@@ -1150,8 +1151,8 @@
       <c r="C15" t="s">
         <v>76</v>
       </c>
-      <c r="D15">
-        <v>14</v>
+      <c r="D15" s="1" t="s">
+        <v>144</v>
       </c>
     </row>
     <row r="16" spans="1:4" x14ac:dyDescent="0.45">
@@ -1164,8 +1165,8 @@
       <c r="C16" t="s">
         <v>77</v>
       </c>
-      <c r="D16">
-        <v>15</v>
+      <c r="D16" s="1" t="s">
+        <v>145</v>
       </c>
     </row>
     <row r="17" spans="1:4" x14ac:dyDescent="0.45">
@@ -1178,8 +1179,8 @@
       <c r="C17" t="s">
         <v>78</v>
       </c>
-      <c r="D17">
-        <v>16</v>
+      <c r="D17" s="1" t="s">
+        <v>146</v>
       </c>
     </row>
     <row r="18" spans="1:4" x14ac:dyDescent="0.45">
@@ -1192,8 +1193,8 @@
       <c r="C18" t="s">
         <v>79</v>
       </c>
-      <c r="D18">
-        <v>17</v>
+      <c r="D18" s="1" t="s">
+        <v>147</v>
       </c>
     </row>
     <row r="19" spans="1:4" x14ac:dyDescent="0.45">
@@ -1206,8 +1207,8 @@
       <c r="C19" t="s">
         <v>80</v>
       </c>
-      <c r="D19">
-        <v>18</v>
+      <c r="D19" s="1" t="s">
+        <v>148</v>
       </c>
     </row>
     <row r="20" spans="1:4" x14ac:dyDescent="0.45">
@@ -1220,8 +1221,8 @@
       <c r="C20" t="s">
         <v>81</v>
       </c>
-      <c r="D20">
-        <v>19</v>
+      <c r="D20" s="1" t="s">
+        <v>149</v>
       </c>
     </row>
     <row r="21" spans="1:4" x14ac:dyDescent="0.45">
@@ -1234,8 +1235,8 @@
       <c r="C21" t="s">
         <v>82</v>
       </c>
-      <c r="D21">
-        <v>20</v>
+      <c r="D21" s="1" t="s">
+        <v>150</v>
       </c>
     </row>
     <row r="22" spans="1:4" x14ac:dyDescent="0.45">
@@ -1248,8 +1249,8 @@
       <c r="C22" t="s">
         <v>83</v>
       </c>
-      <c r="D22">
-        <v>21</v>
+      <c r="D22" s="1" t="s">
+        <v>151</v>
       </c>
     </row>
     <row r="23" spans="1:4" x14ac:dyDescent="0.45">
@@ -1262,8 +1263,8 @@
       <c r="C23" t="s">
         <v>84</v>
       </c>
-      <c r="D23">
-        <v>22</v>
+      <c r="D23" s="1" t="s">
+        <v>152</v>
       </c>
     </row>
     <row r="24" spans="1:4" x14ac:dyDescent="0.45">
@@ -1276,8 +1277,8 @@
       <c r="C24" t="s">
         <v>85</v>
       </c>
-      <c r="D24">
-        <v>23</v>
+      <c r="D24" s="1" t="s">
+        <v>153</v>
       </c>
     </row>
     <row r="25" spans="1:4" x14ac:dyDescent="0.45">
@@ -1290,8 +1291,8 @@
       <c r="C25" t="s">
         <v>86</v>
       </c>
-      <c r="D25">
-        <v>24</v>
+      <c r="D25" s="1" t="s">
+        <v>154</v>
       </c>
     </row>
     <row r="26" spans="1:4" x14ac:dyDescent="0.45">
@@ -1304,8 +1305,8 @@
       <c r="C26" t="s">
         <v>87</v>
       </c>
-      <c r="D26">
-        <v>25</v>
+      <c r="D26" s="1" t="s">
+        <v>155</v>
       </c>
     </row>
     <row r="27" spans="1:4" x14ac:dyDescent="0.45">
@@ -1318,8 +1319,8 @@
       <c r="C27" t="s">
         <v>88</v>
       </c>
-      <c r="D27">
-        <v>26</v>
+      <c r="D27" s="1" t="s">
+        <v>156</v>
       </c>
     </row>
     <row r="28" spans="1:4" x14ac:dyDescent="0.45">
@@ -1332,8 +1333,8 @@
       <c r="C28" t="s">
         <v>89</v>
       </c>
-      <c r="D28">
-        <v>27</v>
+      <c r="D28" s="1" t="s">
+        <v>157</v>
       </c>
     </row>
     <row r="29" spans="1:4" x14ac:dyDescent="0.45">
@@ -1346,8 +1347,8 @@
       <c r="C29" t="s">
         <v>90</v>
       </c>
-      <c r="D29">
-        <v>28</v>
+      <c r="D29" s="1" t="s">
+        <v>158</v>
       </c>
     </row>
     <row r="30" spans="1:4" x14ac:dyDescent="0.45">
@@ -1360,8 +1361,8 @@
       <c r="C30" t="s">
         <v>91</v>
       </c>
-      <c r="D30">
-        <v>29</v>
+      <c r="D30" s="1" t="s">
+        <v>159</v>
       </c>
     </row>
     <row r="31" spans="1:4" x14ac:dyDescent="0.45">
@@ -1374,8 +1375,8 @@
       <c r="C31" t="s">
         <v>92</v>
       </c>
-      <c r="D31">
-        <v>30</v>
+      <c r="D31" s="1" t="s">
+        <v>160</v>
       </c>
     </row>
     <row r="32" spans="1:4" x14ac:dyDescent="0.45">
@@ -1388,8 +1389,8 @@
       <c r="C32" t="s">
         <v>93</v>
       </c>
-      <c r="D32">
-        <v>31</v>
+      <c r="D32" s="1" t="s">
+        <v>161</v>
       </c>
     </row>
     <row r="33" spans="1:4" x14ac:dyDescent="0.45">
@@ -1402,8 +1403,8 @@
       <c r="C33" t="s">
         <v>94</v>
       </c>
-      <c r="D33">
-        <v>32</v>
+      <c r="D33" s="1" t="s">
+        <v>162</v>
       </c>
     </row>
     <row r="34" spans="1:4" x14ac:dyDescent="0.45">
@@ -1416,8 +1417,8 @@
       <c r="C34" t="s">
         <v>95</v>
       </c>
-      <c r="D34">
-        <v>33</v>
+      <c r="D34" s="1" t="s">
+        <v>163</v>
       </c>
     </row>
     <row r="35" spans="1:4" x14ac:dyDescent="0.45">
@@ -1430,8 +1431,8 @@
       <c r="C35" t="s">
         <v>96</v>
       </c>
-      <c r="D35">
-        <v>34</v>
+      <c r="D35" s="1" t="s">
+        <v>164</v>
       </c>
     </row>
     <row r="36" spans="1:4" x14ac:dyDescent="0.45">
@@ -1444,8 +1445,8 @@
       <c r="C36" t="s">
         <v>97</v>
       </c>
-      <c r="D36">
-        <v>35</v>
+      <c r="D36" s="1" t="s">
+        <v>165</v>
       </c>
     </row>
     <row r="37" spans="1:4" x14ac:dyDescent="0.45">
@@ -1458,8 +1459,8 @@
       <c r="C37" t="s">
         <v>98</v>
       </c>
-      <c r="D37">
-        <v>36</v>
+      <c r="D37" s="1" t="s">
+        <v>166</v>
       </c>
     </row>
     <row r="38" spans="1:4" x14ac:dyDescent="0.45">
@@ -1472,8 +1473,8 @@
       <c r="C38" t="s">
         <v>99</v>
       </c>
-      <c r="D38">
-        <v>37</v>
+      <c r="D38" s="1" t="s">
+        <v>167</v>
       </c>
     </row>
     <row r="39" spans="1:4" x14ac:dyDescent="0.45">
@@ -1486,8 +1487,8 @@
       <c r="C39" t="s">
         <v>100</v>
       </c>
-      <c r="D39">
-        <v>38</v>
+      <c r="D39" s="1" t="s">
+        <v>168</v>
       </c>
     </row>
     <row r="40" spans="1:4" x14ac:dyDescent="0.45">
@@ -1500,8 +1501,8 @@
       <c r="C40" t="s">
         <v>101</v>
       </c>
-      <c r="D40">
-        <v>39</v>
+      <c r="D40" s="1" t="s">
+        <v>169</v>
       </c>
     </row>
     <row r="41" spans="1:4" x14ac:dyDescent="0.45">
@@ -1514,8 +1515,8 @@
       <c r="C41" t="s">
         <v>102</v>
       </c>
-      <c r="D41">
-        <v>40</v>
+      <c r="D41" s="1" t="s">
+        <v>170</v>
       </c>
     </row>
     <row r="42" spans="1:4" x14ac:dyDescent="0.45">
@@ -1528,8 +1529,8 @@
       <c r="C42" t="s">
         <v>103</v>
       </c>
-      <c r="D42">
-        <v>41</v>
+      <c r="D42" s="1" t="s">
+        <v>171</v>
       </c>
     </row>
     <row r="43" spans="1:4" x14ac:dyDescent="0.45">
@@ -1542,8 +1543,8 @@
       <c r="C43" t="s">
         <v>104</v>
       </c>
-      <c r="D43">
-        <v>42</v>
+      <c r="D43" s="1" t="s">
+        <v>172</v>
       </c>
     </row>
     <row r="44" spans="1:4" x14ac:dyDescent="0.45">
@@ -1556,8 +1557,8 @@
       <c r="C44" t="s">
         <v>105</v>
       </c>
-      <c r="D44">
-        <v>43</v>
+      <c r="D44" s="1" t="s">
+        <v>173</v>
       </c>
     </row>
     <row r="45" spans="1:4" x14ac:dyDescent="0.45">
@@ -1570,8 +1571,8 @@
       <c r="C45" t="s">
         <v>106</v>
       </c>
-      <c r="D45">
-        <v>44</v>
+      <c r="D45" s="1" t="s">
+        <v>174</v>
       </c>
     </row>
     <row r="46" spans="1:4" x14ac:dyDescent="0.45">
@@ -1584,8 +1585,8 @@
       <c r="C46" t="s">
         <v>107</v>
       </c>
-      <c r="D46">
-        <v>45</v>
+      <c r="D46" s="1" t="s">
+        <v>175</v>
       </c>
     </row>
     <row r="47" spans="1:4" x14ac:dyDescent="0.45">
@@ -1598,8 +1599,8 @@
       <c r="C47" t="s">
         <v>108</v>
       </c>
-      <c r="D47">
-        <v>46</v>
+      <c r="D47" s="1" t="s">
+        <v>176</v>
       </c>
     </row>
     <row r="48" spans="1:4" x14ac:dyDescent="0.45">
@@ -1612,8 +1613,8 @@
       <c r="C48" t="s">
         <v>109</v>
       </c>
-      <c r="D48">
-        <v>47</v>
+      <c r="D48" s="1" t="s">
+        <v>177</v>
       </c>
     </row>
     <row r="49" spans="1:4" x14ac:dyDescent="0.45">
@@ -1626,8 +1627,8 @@
       <c r="C49" t="s">
         <v>110</v>
       </c>
-      <c r="D49">
-        <v>48</v>
+      <c r="D49" s="1" t="s">
+        <v>178</v>
       </c>
     </row>
     <row r="50" spans="1:4" x14ac:dyDescent="0.45">
@@ -1640,8 +1641,8 @@
       <c r="C50" t="s">
         <v>111</v>
       </c>
-      <c r="D50">
-        <v>49</v>
+      <c r="D50" s="1" t="s">
+        <v>179</v>
       </c>
     </row>
     <row r="51" spans="1:4" x14ac:dyDescent="0.45">
@@ -1654,8 +1655,8 @@
       <c r="C51" t="s">
         <v>112</v>
       </c>
-      <c r="D51">
-        <v>50</v>
+      <c r="D51" s="1" t="s">
+        <v>180</v>
       </c>
     </row>
     <row r="52" spans="1:4" x14ac:dyDescent="0.45">
@@ -1668,8 +1669,8 @@
       <c r="C52" t="s">
         <v>113</v>
       </c>
-      <c r="D52">
-        <v>51</v>
+      <c r="D52" s="1" t="s">
+        <v>181</v>
       </c>
     </row>
     <row r="53" spans="1:4" x14ac:dyDescent="0.45">
@@ -1682,8 +1683,8 @@
       <c r="C53" t="s">
         <v>114</v>
       </c>
-      <c r="D53">
-        <v>52</v>
+      <c r="D53" s="1" t="s">
+        <v>182</v>
       </c>
     </row>
     <row r="54" spans="1:4" x14ac:dyDescent="0.45">
@@ -1696,8 +1697,8 @@
       <c r="C54" t="s">
         <v>115</v>
       </c>
-      <c r="D54">
-        <v>53</v>
+      <c r="D54" s="1" t="s">
+        <v>183</v>
       </c>
     </row>
     <row r="55" spans="1:4" x14ac:dyDescent="0.45">
@@ -1710,8 +1711,8 @@
       <c r="C55" t="s">
         <v>116</v>
       </c>
-      <c r="D55">
-        <v>54</v>
+      <c r="D55" s="1" t="s">
+        <v>184</v>
       </c>
     </row>
     <row r="56" spans="1:4" x14ac:dyDescent="0.45">
@@ -1724,8 +1725,8 @@
       <c r="C56" t="s">
         <v>117</v>
       </c>
-      <c r="D56">
-        <v>55</v>
+      <c r="D56" s="1" t="s">
+        <v>185</v>
       </c>
     </row>
     <row r="57" spans="1:4" x14ac:dyDescent="0.45">
@@ -1738,8 +1739,8 @@
       <c r="C57" t="s">
         <v>118</v>
       </c>
-      <c r="D57">
-        <v>56</v>
+      <c r="D57" s="1" t="s">
+        <v>186</v>
       </c>
     </row>
     <row r="58" spans="1:4" x14ac:dyDescent="0.45">
@@ -1752,8 +1753,8 @@
       <c r="C58" t="s">
         <v>119</v>
       </c>
-      <c r="D58">
-        <v>57</v>
+      <c r="D58" s="1" t="s">
+        <v>187</v>
       </c>
     </row>
     <row r="59" spans="1:4" x14ac:dyDescent="0.45">
@@ -1766,8 +1767,8 @@
       <c r="C59" t="s">
         <v>120</v>
       </c>
-      <c r="D59">
-        <v>58</v>
+      <c r="D59" s="1" t="s">
+        <v>188</v>
       </c>
     </row>
     <row r="60" spans="1:4" x14ac:dyDescent="0.45">
@@ -1780,8 +1781,8 @@
       <c r="C60" t="s">
         <v>121</v>
       </c>
-      <c r="D60">
-        <v>59</v>
+      <c r="D60" s="1" t="s">
+        <v>189</v>
       </c>
     </row>
     <row r="61" spans="1:4" x14ac:dyDescent="0.45">
@@ -1794,8 +1795,8 @@
       <c r="C61" t="s">
         <v>122</v>
       </c>
-      <c r="D61">
-        <v>60</v>
+      <c r="D61" s="1" t="s">
+        <v>190</v>
       </c>
     </row>
     <row r="62" spans="1:4" x14ac:dyDescent="0.45">
@@ -1808,8 +1809,8 @@
       <c r="C62" t="s">
         <v>123</v>
       </c>
-      <c r="D62">
-        <v>61</v>
+      <c r="D62" s="1" t="s">
+        <v>191</v>
       </c>
     </row>
     <row r="63" spans="1:4" x14ac:dyDescent="0.45">
@@ -1822,8 +1823,8 @@
       <c r="C63" t="s">
         <v>124</v>
       </c>
-      <c r="D63">
-        <v>62</v>
+      <c r="D63" s="1" t="s">
+        <v>192</v>
       </c>
     </row>
     <row r="64" spans="1:4" x14ac:dyDescent="0.45">
@@ -1836,8 +1837,8 @@
       <c r="C64" t="s">
         <v>125</v>
       </c>
-      <c r="D64">
-        <v>63</v>
+      <c r="D64" s="1" t="s">
+        <v>193</v>
       </c>
     </row>
     <row r="65" spans="1:4" x14ac:dyDescent="0.45">
@@ -1850,8 +1851,8 @@
       <c r="C65" t="s">
         <v>126</v>
       </c>
-      <c r="D65">
-        <v>64</v>
+      <c r="D65" s="1" t="s">
+        <v>194</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Fix Google Drive export/import for Google Sheets/Docs
</commit_message>
<xml_diff>
--- a/DANH SÁCH THÍ SINH.xlsx
+++ b/DANH SÁCH THÍ SINH.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="E:\TAO UNG DUNG\GAME RUNG CHUONG VANG\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{973387B7-B8AD-4AA1-8988-8B6C796DCF03}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{26A46A5A-8AB2-4F19-B555-995E2307FF24}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-98" yWindow="-98" windowWidth="20715" windowHeight="13155" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -423,196 +423,196 @@
     <t>NGUYỄN VĂN NHÀN</t>
   </si>
   <si>
-    <t>101</t>
-  </si>
-  <si>
-    <t>102</t>
-  </si>
-  <si>
-    <t>103</t>
-  </si>
-  <si>
-    <t>104</t>
-  </si>
-  <si>
-    <t>105</t>
-  </si>
-  <si>
-    <t>106</t>
-  </si>
-  <si>
-    <t>107</t>
-  </si>
-  <si>
-    <t>108</t>
-  </si>
-  <si>
-    <t>109</t>
-  </si>
-  <si>
-    <t>110</t>
-  </si>
-  <si>
-    <t>111</t>
-  </si>
-  <si>
-    <t>112</t>
-  </si>
-  <si>
-    <t>113</t>
-  </si>
-  <si>
-    <t>114</t>
-  </si>
-  <si>
-    <t>115</t>
-  </si>
-  <si>
-    <t>116</t>
-  </si>
-  <si>
-    <t>117</t>
-  </si>
-  <si>
-    <t>118</t>
-  </si>
-  <si>
-    <t>119</t>
-  </si>
-  <si>
-    <t>120</t>
-  </si>
-  <si>
-    <t>121</t>
-  </si>
-  <si>
-    <t>122</t>
-  </si>
-  <si>
-    <t>123</t>
-  </si>
-  <si>
-    <t>124</t>
-  </si>
-  <si>
-    <t>125</t>
-  </si>
-  <si>
-    <t>126</t>
-  </si>
-  <si>
-    <t>127</t>
-  </si>
-  <si>
-    <t>128</t>
-  </si>
-  <si>
-    <t>129</t>
-  </si>
-  <si>
-    <t>130</t>
-  </si>
-  <si>
-    <t>131</t>
-  </si>
-  <si>
-    <t>132</t>
-  </si>
-  <si>
-    <t>133</t>
-  </si>
-  <si>
-    <t>134</t>
-  </si>
-  <si>
-    <t>135</t>
-  </si>
-  <si>
-    <t>136</t>
-  </si>
-  <si>
-    <t>137</t>
-  </si>
-  <si>
-    <t>138</t>
-  </si>
-  <si>
-    <t>139</t>
-  </si>
-  <si>
-    <t>140</t>
-  </si>
-  <si>
-    <t>141</t>
-  </si>
-  <si>
-    <t>142</t>
-  </si>
-  <si>
-    <t>143</t>
-  </si>
-  <si>
-    <t>144</t>
-  </si>
-  <si>
-    <t>145</t>
-  </si>
-  <si>
-    <t>146</t>
-  </si>
-  <si>
-    <t>147</t>
-  </si>
-  <si>
-    <t>148</t>
-  </si>
-  <si>
-    <t>149</t>
-  </si>
-  <si>
-    <t>150</t>
-  </si>
-  <si>
-    <t>151</t>
-  </si>
-  <si>
-    <t>152</t>
-  </si>
-  <si>
-    <t>153</t>
-  </si>
-  <si>
-    <t>154</t>
-  </si>
-  <si>
-    <t>155</t>
-  </si>
-  <si>
-    <t>156</t>
-  </si>
-  <si>
-    <t>157</t>
-  </si>
-  <si>
-    <t>158</t>
-  </si>
-  <si>
-    <t>159</t>
-  </si>
-  <si>
-    <t>160</t>
-  </si>
-  <si>
-    <t>161</t>
-  </si>
-  <si>
-    <t>162</t>
-  </si>
-  <si>
-    <t>163</t>
-  </si>
-  <si>
-    <t>164</t>
+    <t>01</t>
+  </si>
+  <si>
+    <t>02</t>
+  </si>
+  <si>
+    <t>03</t>
+  </si>
+  <si>
+    <t>04</t>
+  </si>
+  <si>
+    <t>05</t>
+  </si>
+  <si>
+    <t>06</t>
+  </si>
+  <si>
+    <t>07</t>
+  </si>
+  <si>
+    <t>08</t>
+  </si>
+  <si>
+    <t>09</t>
+  </si>
+  <si>
+    <t>10</t>
+  </si>
+  <si>
+    <t>11</t>
+  </si>
+  <si>
+    <t>12</t>
+  </si>
+  <si>
+    <t>13</t>
+  </si>
+  <si>
+    <t>14</t>
+  </si>
+  <si>
+    <t>15</t>
+  </si>
+  <si>
+    <t>16</t>
+  </si>
+  <si>
+    <t>17</t>
+  </si>
+  <si>
+    <t>18</t>
+  </si>
+  <si>
+    <t>19</t>
+  </si>
+  <si>
+    <t>20</t>
+  </si>
+  <si>
+    <t>21</t>
+  </si>
+  <si>
+    <t>22</t>
+  </si>
+  <si>
+    <t>23</t>
+  </si>
+  <si>
+    <t>24</t>
+  </si>
+  <si>
+    <t>25</t>
+  </si>
+  <si>
+    <t>26</t>
+  </si>
+  <si>
+    <t>27</t>
+  </si>
+  <si>
+    <t>28</t>
+  </si>
+  <si>
+    <t>29</t>
+  </si>
+  <si>
+    <t>30</t>
+  </si>
+  <si>
+    <t>31</t>
+  </si>
+  <si>
+    <t>32</t>
+  </si>
+  <si>
+    <t>33</t>
+  </si>
+  <si>
+    <t>34</t>
+  </si>
+  <si>
+    <t>35</t>
+  </si>
+  <si>
+    <t>36</t>
+  </si>
+  <si>
+    <t>37</t>
+  </si>
+  <si>
+    <t>38</t>
+  </si>
+  <si>
+    <t>39</t>
+  </si>
+  <si>
+    <t>40</t>
+  </si>
+  <si>
+    <t>41</t>
+  </si>
+  <si>
+    <t>42</t>
+  </si>
+  <si>
+    <t>43</t>
+  </si>
+  <si>
+    <t>44</t>
+  </si>
+  <si>
+    <t>45</t>
+  </si>
+  <si>
+    <t>46</t>
+  </si>
+  <si>
+    <t>47</t>
+  </si>
+  <si>
+    <t>48</t>
+  </si>
+  <si>
+    <t>49</t>
+  </si>
+  <si>
+    <t>50</t>
+  </si>
+  <si>
+    <t>51</t>
+  </si>
+  <si>
+    <t>52</t>
+  </si>
+  <si>
+    <t>53</t>
+  </si>
+  <si>
+    <t>54</t>
+  </si>
+  <si>
+    <t>55</t>
+  </si>
+  <si>
+    <t>56</t>
+  </si>
+  <si>
+    <t>57</t>
+  </si>
+  <si>
+    <t>58</t>
+  </si>
+  <si>
+    <t>59</t>
+  </si>
+  <si>
+    <t>60</t>
+  </si>
+  <si>
+    <t>61</t>
+  </si>
+  <si>
+    <t>62</t>
+  </si>
+  <si>
+    <t>63</t>
+  </si>
+  <si>
+    <t>64</t>
   </si>
 </sst>
 </file>

</xml_diff>